<commit_message>
Add landscaping CPO presentation and updated drinking water analysis outputs
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/spend-analysis/outputs/DRINKING_WATER_PILOT_ANALYSIS_WORKBOOK.xlsx
+++ b/spend-analysis/outputs/DRINKING_WATER_PILOT_ANALYSIS_WORKBOOK.xlsx
@@ -28,7 +28,7 @@
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -55,8 +55,37 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -81,6 +110,24 @@
         <bgColor rgb="00D9EAD3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000071BC"/>
+        <bgColor rgb="000071BC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F4FD"/>
+        <bgColor rgb="00E8F4FD"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -100,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -118,6 +165,46 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -484,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -550,7 +637,7 @@
           <t>Total Transactions</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B8" s="7" t="n">
         <v>240</v>
       </c>
     </row>
@@ -560,7 +647,7 @@
           <t>Total Vendors</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B9" s="7" t="n">
         <v>4</v>
       </c>
     </row>
@@ -570,7 +657,7 @@
           <t>Total Departments (Using Areas)</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B10" s="7" t="n">
         <v>13</v>
       </c>
     </row>
@@ -616,14 +703,26 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>Projected Annual Benefit Range:</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>$11,353 - $20,907</t>
+      <c r="B17" s="15" t="inlineStr">
+        <is>
+          <t>$18,357 - $24,311</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>3-Year Projected Value:</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>$55,071 - $72,933</t>
         </is>
       </c>
     </row>
@@ -1269,12 +1368,6 @@
           <t>FRAGMENTATION SUMMARY</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1287,11 +1380,6 @@
           <t>51-Public Safety Admin, 57-Chicago Police</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1304,11 +1392,6 @@
           <t>59-Chicago Fire</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1321,11 +1404,6 @@
           <t>10 departments (all others)</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1857,14 +1935,11 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
           <t>WHY ANNUALIZE FIRST?</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" s="13" t="inlineStr">
         <is>
           <t>We annualize BEFORE applying savings rates because we are projecting forward-looking annual savings from FUTURE contracts, not retroactive savings on historical spend. The 5-year data establishes the annual run rate baseline. Savings come from contracts we negotiate going forward.</t>
@@ -1886,7 +1961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1937,10 +2012,8 @@
           <t>Conservative</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>5%</t>
-        </is>
+      <c r="B6" s="14" t="n">
+        <v>0.05</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -1957,10 +2030,8 @@
           <t>Moderate (RECOMMENDED)</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>10%</t>
-        </is>
+      <c r="B7" s="14" t="n">
+        <v>0.1</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1977,10 +2048,8 @@
           <t>Aggressive</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
+      <c r="B8" s="14" t="n">
+        <v>0.15</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -2041,7 +2110,6 @@
           <t>$700,404.52 ÷ 5</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
       <c r="D16" s="5" t="n">
         <v>140080.904</v>
       </c>
@@ -2057,7 +2125,6 @@
           <t>BLS Producer Price Index</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
       <c r="D17" s="6" t="n">
         <v>0.05</v>
       </c>
@@ -2073,7 +2140,6 @@
           <t>$140,080.90 × 5%</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
       <c r="D18" s="5" t="n">
         <v>7004.0452</v>
       </c>
@@ -2121,7 +2187,6 @@
           <t>240 ÷ 5</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
       <c r="D25" s="7" t="n">
         <v>48</v>
       </c>
@@ -2137,7 +2202,6 @@
           <t>12 (quarterly per vendor)</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
       <c r="D26" s="7" t="n">
         <v>12</v>
       </c>
@@ -2153,7 +2217,6 @@
           <t>48 - 12</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
       <c r="D27" s="7" t="n">
         <v>36</v>
       </c>
@@ -2169,8 +2232,6 @@
           <t>$150 - $250</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2183,7 +2244,6 @@
           <t>36 × $150 to 36 × $250</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
           <t>$5,400 - $9,000</t>
@@ -2205,17 +2265,17 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+      <c r="A35" s="26" t="inlineStr">
         <is>
           <t>Benefit Type</t>
         </is>
       </c>
-      <c r="B35" s="4" t="inlineStr">
+      <c r="B35" s="27" t="inlineStr">
         <is>
           <t>Conservative</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr">
+      <c r="C35" s="27" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
@@ -2223,60 +2283,69 @@
       <c r="D35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Consolidation Savings</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="n">
+      <c r="A36" s="19" t="inlineStr">
+        <is>
+          <t>Hard Cost Savings (Consolidation)</t>
+        </is>
+      </c>
+      <c r="B36" s="20" t="n">
         <v>5953</v>
       </c>
-      <c r="C36" s="5" t="n">
+      <c r="C36" s="20" t="n">
         <v>11907</v>
       </c>
-      <c r="D36" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Admin Savings (low)</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="n">
+      <c r="A37" s="21" t="inlineStr">
+        <is>
+          <t>Cost Avoidance (Inflation @ 5% BLS PPI)</t>
+        </is>
+      </c>
+      <c r="B37" s="22" t="n">
+        <v>7004</v>
+      </c>
+      <c r="C37" s="22" t="n">
+        <v>7004</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="21" t="inlineStr">
+        <is>
+          <t>Admin Savings (36 fewer transactions @ $150)</t>
+        </is>
+      </c>
+      <c r="B38" s="22" t="n">
         <v>5400</v>
       </c>
-      <c r="C37" s="5" t="n">
+      <c r="C38" s="22" t="n">
         <v>5400</v>
       </c>
-      <c r="D37" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="3" t="inlineStr">
+    </row>
+    <row r="39">
+      <c r="A39" s="23" t="inlineStr">
         <is>
           <t>Annual Total</t>
         </is>
       </c>
-      <c r="B38" s="12" t="n">
-        <v>11353</v>
-      </c>
-      <c r="C38" s="12" t="n">
-        <v>17307</v>
-      </c>
-      <c r="D38" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
+      <c r="B39" s="24" t="n">
+        <v>18357</v>
+      </c>
+      <c r="C39" s="24" t="n">
+        <v>24311</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="16" t="inlineStr">
         <is>
           <t>3-Year Total</t>
         </is>
       </c>
-      <c r="B39" s="12" t="n">
-        <v>34060</v>
-      </c>
-      <c r="C39" s="12" t="n">
-        <v>51920</v>
-      </c>
-      <c r="D39" t="inlineStr"/>
+      <c r="B40" s="25" t="n">
+        <v>55071</v>
+      </c>
+      <c r="C40" s="25" t="n">
+        <v>72933</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -2597,7 +2666,6 @@
           <t>EY projected $55M-$111M in citywide savings through Category Management. This pilot applies the SAME methodology to the simplest possible category to prove the model before scaling. If consolidation works for drinking water (zero risk, clear commodity), it validates the approach for higher-value categories and the broader vendor tail.</t>
         </is>
       </c>
-      <c r="B16" s="13" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>